<commit_message>
feat(import): Chevening scholar, cohort, university and CAM member
Optional import columns, stored as the website form stores them
('Yes'/'No' with cohort and university), so imported people show them in
View details and the registrations export. A yes/no column holding
anything else is reported for that row. Templates and example updated.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/frontend/public/samples/attendees-template.xlsx
+++ b/frontend/public/samples/attendees-template.xlsx
@@ -67,17 +67,21 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F1"/>
+  <dimension ref="A1:J1"/>
   <cols>
     <col min="1" max="1" width="28" customWidth="true"/>
     <col min="2" max="2" width="34" customWidth="true"/>
     <col min="3" max="3" width="20" customWidth="true"/>
     <col min="4" max="4" width="34" customWidth="true"/>
     <col min="5" max="5" width="28" customWidth="true"/>
-    <col min="6" max="6" width="12" customWidth="true"/>
+    <col min="6" max="6" width="20" customWidth="true"/>
+    <col min="7" max="7" width="18" customWidth="true"/>
+    <col min="8" max="8" width="34" customWidth="true"/>
+    <col min="9" max="9" width="14" customWidth="true"/>
+    <col min="10" max="10" width="12" customWidth="true"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" customHeight="0">
+    <row r="1" spans="1:10" customHeight="0">
       <c r="A1" s="1" t="inlineStr">
         <is>
           <t>name</t>
@@ -105,6 +109,26 @@
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
+          <t>chevening_scholar</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>chevening_cohort</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>chevening_university</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>cam_member</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
           <t>arrived</t>
         </is>
       </c>

</xml_diff>